<commit_message>
AP-07: Daten Jahrgang 6 und 7 uebertragen
Jg6.xlsx: 25 Slots inkl. Sonderwochen und Bausteine, Jg7.xlsx: 21 Slots
(einschliesslich jg7-fvu-1, faecherverbindender Unterricht ueber alle drei
Spuren). Titel aus anhang/slots_2026-27.json uebernommen, leere Titel
("Thema folgt") bewusst so belassen, wo die Quelle keinen Titel angibt
(Jg6: en-5/geo-5; Jg7: alle ausser fvu-1, laut Leo "erstmal offen lassen").
tools/fill_jg6.mjs, tools/fill_jg7.mjs sind die wiederholbaren
Erzeugungsskripte dazu (wie fill_jg5.mjs aus AP-06).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg6.xlsx
+++ b/content/jahrgaenge/Jg6.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="219">
   <si>
     <t>Hinweise zu Jg6.xlsx</t>
   </si>
@@ -497,14 +497,195 @@
   </si>
   <si>
     <t>Bausteinzeitraum 31.08. bis 02.10.2026</t>
+  </si>
+  <si>
+    <t>klar</t>
+  </si>
+  <si>
+    <t>Besinn-Dich-Tage</t>
+  </si>
+  <si>
+    <t>besinntage</t>
+  </si>
+  <si>
+    <t>letzte Schulwoche</t>
+  </si>
+  <si>
+    <t>letzte-woche</t>
+  </si>
+  <si>
+    <t>jg6-de-1</t>
+  </si>
+  <si>
+    <t>jg6-ma-1</t>
+  </si>
+  <si>
+    <t>ma</t>
+  </si>
+  <si>
+    <t>jg6-bio-1</t>
+  </si>
+  <si>
+    <t>jg6-en-1</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>jg6-geo-1</t>
+  </si>
+  <si>
+    <t>geo</t>
+  </si>
+  <si>
+    <t>jg6-ma-2</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>jg6-de-2</t>
+  </si>
+  <si>
+    <t>jg6-bio-2</t>
+  </si>
+  <si>
+    <t>jg6-en-2</t>
+  </si>
+  <si>
+    <t>jg6-geo-2</t>
+  </si>
+  <si>
+    <t>jg6-bio-3</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>jg6-ma-3</t>
+  </si>
+  <si>
+    <t>jg6-de-3</t>
+  </si>
+  <si>
+    <t>wahl</t>
+  </si>
+  <si>
+    <t>jg6-en-3</t>
+  </si>
+  <si>
+    <t>jg6-geo-3</t>
+  </si>
+  <si>
+    <t>jg6-en-4</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>jg6-ma-4</t>
+  </si>
+  <si>
+    <t>jg6-bio-4</t>
+  </si>
+  <si>
+    <t>jg6-de-4</t>
+  </si>
+  <si>
+    <t>jg6-geo-4</t>
+  </si>
+  <si>
+    <t>jg6-de-5</t>
+  </si>
+  <si>
+    <t>jg6-ma-5</t>
+  </si>
+  <si>
+    <t>jg6-bio-5</t>
+  </si>
+  <si>
+    <t>jg6-en-5</t>
+  </si>
+  <si>
+    <t>jg6-geo-5</t>
+  </si>
+  <si>
+    <t>Satzglieder</t>
+  </si>
+  <si>
+    <t>Zuordnungen</t>
+  </si>
+  <si>
+    <t>Wirbellose Tiere in ihren Lebensräumen</t>
+  </si>
+  <si>
+    <t>The Secret of Maple Hill</t>
+  </si>
+  <si>
+    <t>Europa</t>
+  </si>
+  <si>
+    <t>Konstruieren von Dreiecken</t>
+  </si>
+  <si>
+    <t>Fabeln</t>
+  </si>
+  <si>
+    <t>Unter der Lupe</t>
+  </si>
+  <si>
+    <t>Christmas</t>
+  </si>
+  <si>
+    <t>Klima in Europa</t>
+  </si>
+  <si>
+    <t>Der Wald als Lebensgemeinschaft</t>
+  </si>
+  <si>
+    <t>weitere Dreieckseigenschaften und Vierecksberechnung</t>
+  </si>
+  <si>
+    <t>Ocean City ODER Herr der Diebe</t>
+  </si>
+  <si>
+    <t>Peacemakers</t>
+  </si>
+  <si>
+    <t>Nordeuropa</t>
+  </si>
+  <si>
+    <t>Pip and the Umbrella Room</t>
+  </si>
+  <si>
+    <t>Eigenschaften und Darstellen von Prismen</t>
+  </si>
+  <si>
+    <t>Samenpflanzen</t>
+  </si>
+  <si>
+    <t>Beschreiben und Berichten</t>
+  </si>
+  <si>
+    <t>Südeuropa</t>
+  </si>
+  <si>
+    <t>Redewendungen und Sprichwörter</t>
+  </si>
+  <si>
+    <t>Volumen von Prismen</t>
+  </si>
+  <si>
+    <t>Exkursionen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -542,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -557,6 +738,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1925,7 +2107,7 @@
     <mergeCell ref="B72:D72"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1956,7 +2138,7 @@
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1992,6 +2174,9 @@
       <c r="A2">
         <v>6</v>
       </c>
+      <c r="B2" t="s">
+        <v>159</v>
+      </c>
       <c r="C2" t="s">
         <v>17</v>
       </c>
@@ -2000,19 +2185,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"verspielt,klar,sachlich"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"verspielt,klar,sachlich"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="13" style="5" customWidth="1"/>
@@ -2034,21 +2222,66 @@
         <v>34</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B2" s="8">
+        <v>46283</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>46468</v>
+      </c>
+      <c r="B3" s="8">
+        <v>46472</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>46573</v>
+      </c>
+      <c r="B4" s="8">
+        <v>46577</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" t="s">
+        <v>163</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="D10:D500">
+      <formula1>"themenwoche,soul-basics,puffer,kennenlernen,einfuehrung,besinntage,fvu,letzte-woche,sonstiges"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:D500">
       <formula1>"themenwoche,soul-basics,puffer,kennenlernen,einfuehrung,besinntage,fvu,letzte-woche,sonstiges"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2099,24 +2332,980 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>16</v>
+      </c>
+      <c r="G2" s="8">
+        <v>46251</v>
+      </c>
+      <c r="H2" s="8">
+        <v>46325</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" t="s">
+        <v>164</v>
+      </c>
+      <c r="K2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>16</v>
+      </c>
+      <c r="G3" s="8">
+        <v>46251</v>
+      </c>
+      <c r="H3" s="8">
+        <v>46276</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" t="s">
+        <v>165</v>
+      </c>
+      <c r="K3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4">
+        <v>16</v>
+      </c>
+      <c r="G4" s="8">
+        <v>46251</v>
+      </c>
+      <c r="H4" s="8">
+        <v>46276</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
+        <v>167</v>
+      </c>
+      <c r="K4" t="s">
+        <v>65</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5">
+        <v>16</v>
+      </c>
+      <c r="G5" s="8">
+        <v>46286</v>
+      </c>
+      <c r="H5" s="8">
+        <v>46325</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" t="s">
+        <v>168</v>
+      </c>
+      <c r="K5" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>16</v>
+      </c>
+      <c r="G6" s="8">
+        <v>46286</v>
+      </c>
+      <c r="H6" s="8">
+        <v>46325</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" t="s">
+        <v>170</v>
+      </c>
+      <c r="K6" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>16</v>
+      </c>
+      <c r="G7" s="8">
+        <v>46328</v>
+      </c>
+      <c r="H7" s="8">
+        <v>46395</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" t="s">
+        <v>172</v>
+      </c>
+      <c r="K7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8">
+        <v>16</v>
+      </c>
+      <c r="G8" s="8">
+        <v>46328</v>
+      </c>
+      <c r="H8" s="8">
+        <v>46353</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J8" t="s">
+        <v>174</v>
+      </c>
+      <c r="K8" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9">
+        <v>16</v>
+      </c>
+      <c r="G9" s="8">
+        <v>46328</v>
+      </c>
+      <c r="H9" s="8">
+        <v>46353</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J9" t="s">
+        <v>175</v>
+      </c>
+      <c r="K9" t="s">
+        <v>65</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10">
+        <v>16</v>
+      </c>
+      <c r="G10" s="8">
+        <v>46356</v>
+      </c>
+      <c r="H10" s="8">
+        <v>46395</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J10" t="s">
+        <v>176</v>
+      </c>
+      <c r="K10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11" t="s">
+        <v>173</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11">
+        <v>16</v>
+      </c>
+      <c r="G11" s="8">
+        <v>46356</v>
+      </c>
+      <c r="H11" s="8">
+        <v>46395</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J11" t="s">
+        <v>177</v>
+      </c>
+      <c r="K11" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12">
+        <v>16</v>
+      </c>
+      <c r="G12" s="8">
+        <v>46398</v>
+      </c>
+      <c r="H12" s="8">
+        <v>46465</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J12" t="s">
+        <v>178</v>
+      </c>
+      <c r="K12" t="s">
+        <v>65</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" t="s">
+        <v>179</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13">
+        <v>16</v>
+      </c>
+      <c r="G13" s="8">
+        <v>46398</v>
+      </c>
+      <c r="H13" s="8">
+        <v>46423</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J13" t="s">
+        <v>180</v>
+      </c>
+      <c r="K13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14">
+        <v>16</v>
+      </c>
+      <c r="G14" s="8">
+        <v>46398</v>
+      </c>
+      <c r="H14" s="8">
+        <v>46423</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J14" t="s">
+        <v>181</v>
+      </c>
+      <c r="K14" t="s">
+        <v>182</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>183</v>
+      </c>
+      <c r="B15" t="s">
+        <v>169</v>
+      </c>
+      <c r="C15" t="s">
+        <v>179</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15">
+        <v>16</v>
+      </c>
+      <c r="G15" s="8">
+        <v>46440</v>
+      </c>
+      <c r="H15" s="8">
+        <v>46465</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J15" t="s">
+        <v>183</v>
+      </c>
+      <c r="K15" t="s">
+        <v>65</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" t="s">
+        <v>171</v>
+      </c>
+      <c r="C16" t="s">
+        <v>179</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16">
+        <v>16</v>
+      </c>
+      <c r="G16" s="8">
+        <v>46440</v>
+      </c>
+      <c r="H16" s="8">
+        <v>46465</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J16" t="s">
+        <v>184</v>
+      </c>
+      <c r="K16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17">
+        <v>16</v>
+      </c>
+      <c r="G17" s="8">
+        <v>46482</v>
+      </c>
+      <c r="H17" s="8">
+        <v>46542</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J17" t="s">
+        <v>185</v>
+      </c>
+      <c r="K17" t="s">
+        <v>65</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" t="s">
+        <v>166</v>
+      </c>
+      <c r="C18" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18">
+        <v>16</v>
+      </c>
+      <c r="G18" s="8">
+        <v>46482</v>
+      </c>
+      <c r="H18" s="8">
+        <v>46507</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" t="s">
+        <v>187</v>
+      </c>
+      <c r="K18" t="s">
+        <v>65</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19">
+        <v>16</v>
+      </c>
+      <c r="G19" s="8">
+        <v>46482</v>
+      </c>
+      <c r="H19" s="8">
+        <v>46507</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" t="s">
+        <v>188</v>
+      </c>
+      <c r="K19" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>186</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20">
+        <v>16</v>
+      </c>
+      <c r="G20" s="8">
+        <v>46510</v>
+      </c>
+      <c r="H20" s="8">
+        <v>46542</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J20" t="s">
+        <v>189</v>
+      </c>
+      <c r="K20" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" t="s">
+        <v>171</v>
+      </c>
+      <c r="C21" t="s">
+        <v>186</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21">
+        <v>16</v>
+      </c>
+      <c r="G21" s="8">
+        <v>46510</v>
+      </c>
+      <c r="H21" s="8">
+        <v>46542</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J21" t="s">
+        <v>190</v>
+      </c>
+      <c r="K21" t="s">
+        <v>65</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22">
+        <v>8</v>
+      </c>
+      <c r="G22" s="8">
+        <v>46545</v>
+      </c>
+      <c r="H22" s="8">
+        <v>46570</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J22" t="s">
+        <v>191</v>
+      </c>
+      <c r="K22" t="s">
+        <v>65</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23">
+        <v>8</v>
+      </c>
+      <c r="G23" s="8">
+        <v>46545</v>
+      </c>
+      <c r="H23" s="8">
+        <v>46556</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J23" t="s">
+        <v>192</v>
+      </c>
+      <c r="K23" t="s">
+        <v>65</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24">
+        <v>8</v>
+      </c>
+      <c r="G24" s="8">
+        <v>46545</v>
+      </c>
+      <c r="H24" s="8">
+        <v>46556</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J24" t="s">
+        <v>193</v>
+      </c>
+      <c r="K24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25">
+        <v>8</v>
+      </c>
+      <c r="G25" s="8">
+        <v>46559</v>
+      </c>
+      <c r="H25" s="8">
+        <v>46570</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" t="s">
+        <v>194</v>
+      </c>
+      <c r="K25" t="s">
+        <v>65</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" t="s">
+        <v>171</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26">
+        <v>3</v>
+      </c>
+      <c r="E26" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26">
+        <v>8</v>
+      </c>
+      <c r="G26" s="8">
+        <v>46559</v>
+      </c>
+      <c r="H26" s="8">
+        <v>46570</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J26" t="s">
+        <v>195</v>
+      </c>
+      <c r="K26" t="s">
+        <v>65</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="K10:K500">
+      <formula1>"fest,wahl,vorlaeufig,offen"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="K2:K500">
       <formula1>"fest,wahl,vorlaeufig,offen"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2155,15 +3344,668 @@
         <v>85</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>183</v>
+      </c>
+      <c r="B15" t="s">
+        <v>169</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" t="s">
+        <v>171</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" t="s">
+        <v>166</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" t="s">
+        <v>171</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" t="s">
+        <v>8</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" t="s">
+        <v>171</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2208,13 +4050,16 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="D10:D500">
+      <formula1>"pflicht,wahl"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:D500">
       <formula1>"pflicht,wahl"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2255,19 +4100,28 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
-  <dataValidations count="3">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C10:C500">
+      <formula1>"fach,methode,baustein"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C2:C500">
       <formula1>"fach,methode,baustein"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F10:F500">
+      <formula1>"ja,nein"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F2:F500">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2300,16 +4154,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="A10:A500">
+      <formula1>"Mo,Di,Mi,Do,Fr"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="A2:A500">
       <formula1>"Mo,Di,Mi,Do,Fr"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="E10:E500">
+      <formula1>"A,B,C"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E2:E500">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2361,21 +4221,33 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
-  <dataValidations count="4">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"input,coaching,sonstiges,entfall"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"input,coaching,sonstiges,entfall"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C10:C500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C2:C500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="E10:E500">
+      <formula1>"A,B,C"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E2:E500">
       <formula1>"A,B,C"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I10:I500">
+      <formula1>"ja,nein"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="I2:I500">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Jg6 Zeitraum 2: Stationen und Gelingensnachweis aus den PDFs eingetragen
Leo hat die Uebersichten fuer Deutsch (Satzglieder), Englisch (The
Secret of Maple Hill) und Geografie (Europa) geschickt. Slots und
Bausteine-Titel standen schon richtig drin, es fehlten die 42
Stationen (Titel, Pflicht/Wahl, Zeit, Niveau, Material) und die
Gelingensnachweis-Angaben. Termine (Inputs/Coachings) und der
"Paedagogische Tag" am 26.10. folgen separat - dafuer fehlt noch eine
Antwort, ob Letzterer schulweit als Ferientag gilt.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg6.xlsx
+++ b/content/jahrgaenge/Jg6.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="298">
   <si>
     <t>Hinweise zu Jg6.xlsx</t>
   </si>
@@ -613,6 +613,9 @@
     <t>Satzglieder</t>
   </si>
   <si>
+    <t>Lernübersicht zur Grammatik</t>
+  </si>
+  <si>
     <t>Zuordnungen</t>
   </si>
   <si>
@@ -622,9 +625,15 @@
     <t>The Secret of Maple Hill</t>
   </si>
   <si>
+    <t>report on the events of the story – graded task</t>
+  </si>
+  <si>
     <t>Europa</t>
   </si>
   <si>
+    <t>Klimadiagramm zeichnen</t>
+  </si>
+  <si>
     <t>Konstruieren von Dreiecken</t>
   </si>
   <si>
@@ -677,6 +686,234 @@
   </si>
   <si>
     <t>Exkursionen</t>
+  </si>
+  <si>
+    <t>Sätze würfeln</t>
+  </si>
+  <si>
+    <t>M1, Satzgliedwürfel</t>
+  </si>
+  <si>
+    <t>Wiederholung aller Satzglieder</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>Der Hauptsatz</t>
+  </si>
+  <si>
+    <t>A1, Laptop</t>
+  </si>
+  <si>
+    <t>Der Nebensatz</t>
+  </si>
+  <si>
+    <t>A2, M2, Laptop</t>
+  </si>
+  <si>
+    <t>Einfache Satzreihen und Satzgefüge</t>
+  </si>
+  <si>
+    <t>A3, Laptop</t>
+  </si>
+  <si>
+    <t>Mehrgliedrige Satzgefüge</t>
+  </si>
+  <si>
+    <t>A4, Laptop</t>
+  </si>
+  <si>
+    <t>Satzbilder zeichnen</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>Zeichensetzung bei wörtlicher Rede</t>
+  </si>
+  <si>
+    <t>M3, Laptop</t>
+  </si>
+  <si>
+    <t>Begleitsätze bei wörtlicher Rede</t>
+  </si>
+  <si>
+    <t>A6, A7</t>
+  </si>
+  <si>
+    <t>Anwendung grammatischer Verfahren</t>
+  </si>
+  <si>
+    <t>A8, Laptop</t>
+  </si>
+  <si>
+    <t>Das kann ich jetzt!</t>
+  </si>
+  <si>
+    <t>M4, Material zur Gestaltung</t>
+  </si>
+  <si>
+    <t>Weiterführende Übungen</t>
+  </si>
+  <si>
+    <t>Welcome to Maple Hill</t>
+  </si>
+  <si>
+    <t>M1</t>
+  </si>
+  <si>
+    <t>Falling Leaves &amp; First Feelings</t>
+  </si>
+  <si>
+    <t>M2, white paper</t>
+  </si>
+  <si>
+    <t>The Strange Note</t>
+  </si>
+  <si>
+    <t>A1, A2, or A3</t>
+  </si>
+  <si>
+    <t>The Poem in the Attic</t>
+  </si>
+  <si>
+    <t>A4, M2, white paper</t>
+  </si>
+  <si>
+    <t>What's Inside?</t>
+  </si>
+  <si>
+    <t>sensory boxes</t>
+  </si>
+  <si>
+    <t>The Mysterious Message</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>A Quiet Day</t>
+  </si>
+  <si>
+    <t>M4</t>
+  </si>
+  <si>
+    <t>Whispers in the Wind</t>
+  </si>
+  <si>
+    <t>laptop, headphones</t>
+  </si>
+  <si>
+    <t>Maple Hill Side-Quests</t>
+  </si>
+  <si>
+    <t>A5, A6, A7, A8</t>
+  </si>
+  <si>
+    <t>Through the Trees</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>The Hidden Door</t>
+  </si>
+  <si>
+    <t>Escape the Forest</t>
+  </si>
+  <si>
+    <t>Between Truth and Silence</t>
+  </si>
+  <si>
+    <t>A9</t>
+  </si>
+  <si>
+    <t>Corinne's Choice – Your Task</t>
+  </si>
+  <si>
+    <t>M5, M6, or M7</t>
+  </si>
+  <si>
+    <t>A Quiet Voice Speaks</t>
+  </si>
+  <si>
+    <t>The Book with Her Name</t>
+  </si>
+  <si>
+    <t>Warm Up</t>
+  </si>
+  <si>
+    <t>A1, Hefter, Stift</t>
+  </si>
+  <si>
+    <t>Länder Europas</t>
+  </si>
+  <si>
+    <t>Atlas, A2, Lehrbuch, Hefter, Stift, Lineal</t>
+  </si>
+  <si>
+    <t>Inseln, Halbinseln, Flüsse, Gebirge Europas</t>
+  </si>
+  <si>
+    <t>A3, A4, Lehrbuch, Atlas, Heft</t>
+  </si>
+  <si>
+    <t>Europa – unser Heimatkontinent</t>
+  </si>
+  <si>
+    <t>Lehrbuch, M1, A5, Heft, Schere, Kleber</t>
+  </si>
+  <si>
+    <t>Großlandschaften Europas</t>
+  </si>
+  <si>
+    <t>Lehrbuch, Heft, A6, M2, Transparentpapier</t>
+  </si>
+  <si>
+    <t>Die Europäische Union</t>
+  </si>
+  <si>
+    <t>Lehrbuch, M3, Heft, Münzen</t>
+  </si>
+  <si>
+    <t>Ländersteckbrief</t>
+  </si>
+  <si>
+    <t>Lehrbuch, A7</t>
+  </si>
+  <si>
+    <t>Wetter und Klima / Klimadiagramm</t>
+  </si>
+  <si>
+    <t>M4, Lehrbuch, A8</t>
+  </si>
+  <si>
+    <t>Klimadiagramm auswerten</t>
+  </si>
+  <si>
+    <t>A9, A10, M4</t>
+  </si>
+  <si>
+    <t>Lehrbuch, kariertes Papier, Millimeterpapier</t>
+  </si>
+  <si>
+    <t>Gelingensnachweis</t>
+  </si>
+  <si>
+    <t>A11, Lehrbuch, Millimeterpapier</t>
+  </si>
+  <si>
+    <t>Universelles Klimadiagramm</t>
+  </si>
+  <si>
+    <t>Pappe, Stecknadeln</t>
+  </si>
+  <si>
+    <t>Vertiefung Topografie</t>
+  </si>
+  <si>
+    <t>A2, A3, A4, Atlas, Wandkarte</t>
   </si>
 </sst>
 </file>
@@ -3358,7 +3595,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>8</v>
+        <v>197</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -3378,7 +3615,7 @@
         <v>166</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>8</v>
@@ -3404,7 +3641,7 @@
         <v>72</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
@@ -3430,16 +3667,16 @@
         <v>169</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
-        <v>8</v>
+        <v>201</v>
+      </c>
+      <c r="F5">
+        <v>15</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>8</v>
@@ -3456,16 +3693,16 @@
         <v>171</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>8</v>
+        <v>203</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>8</v>
@@ -3482,7 +3719,7 @@
         <v>166</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
@@ -3508,7 +3745,7 @@
         <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>8</v>
@@ -3534,7 +3771,7 @@
         <v>72</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>8</v>
@@ -3560,7 +3797,7 @@
         <v>169</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>8</v>
@@ -3586,7 +3823,7 @@
         <v>171</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>8</v>
@@ -3612,7 +3849,7 @@
         <v>72</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>8</v>
@@ -3638,7 +3875,7 @@
         <v>166</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>8</v>
@@ -3664,10 +3901,10 @@
         <v>44</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>8</v>
@@ -3690,7 +3927,7 @@
         <v>169</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>8</v>
@@ -3716,7 +3953,7 @@
         <v>171</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>8</v>
@@ -3742,7 +3979,7 @@
         <v>169</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>8</v>
@@ -3768,7 +4005,7 @@
         <v>166</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>8</v>
@@ -3794,7 +4031,7 @@
         <v>72</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>8</v>
@@ -3820,7 +4057,7 @@
         <v>44</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>8</v>
@@ -3846,7 +4083,7 @@
         <v>171</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>8</v>
@@ -3872,7 +4109,7 @@
         <v>44</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>8</v>
@@ -3898,7 +4135,7 @@
         <v>166</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>8</v>
@@ -3924,7 +4161,7 @@
         <v>72</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>8</v>
@@ -4011,7 +4248,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4046,6 +4283,1098 @@
       </c>
       <c r="H1" s="7" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2">
+        <v>45</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E3">
+        <v>45</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4">
+        <v>45</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5">
+        <v>60</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6">
+        <v>45</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E7">
+        <v>45</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E9">
+        <v>30</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11">
+        <v>45</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D12" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12">
+        <v>80</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D13" t="s">
+        <v>182</v>
+      </c>
+      <c r="E13">
+        <v>60</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D14" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14">
+        <v>60</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15">
+        <v>60</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>168</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D16" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16">
+        <v>30</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>168</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>168</v>
+      </c>
+      <c r="B18">
+        <v>5</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>168</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D19" t="s">
+        <v>93</v>
+      </c>
+      <c r="E19">
+        <v>35</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D20" t="s">
+        <v>182</v>
+      </c>
+      <c r="E20">
+        <v>60</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21">
+        <v>45</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>168</v>
+      </c>
+      <c r="B22">
+        <v>9</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D22" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22">
+        <v>80</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>168</v>
+      </c>
+      <c r="B23">
+        <v>10</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23">
+        <v>35</v>
+      </c>
+      <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24">
+        <v>11</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="D24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24">
+        <v>60</v>
+      </c>
+      <c r="F24">
+        <v>3</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>168</v>
+      </c>
+      <c r="B25">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D25" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25">
+        <v>60</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>168</v>
+      </c>
+      <c r="B26">
+        <v>13</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E26">
+        <v>20</v>
+      </c>
+      <c r="F26">
+        <v>3</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>168</v>
+      </c>
+      <c r="B27">
+        <v>14</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D27" t="s">
+        <v>93</v>
+      </c>
+      <c r="E27">
+        <v>40</v>
+      </c>
+      <c r="F27">
+        <v>3</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B28">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28">
+        <v>100</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>168</v>
+      </c>
+      <c r="B29">
+        <v>16</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D29" t="s">
+        <v>182</v>
+      </c>
+      <c r="E29">
+        <v>25</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>168</v>
+      </c>
+      <c r="B30">
+        <v>17</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D30" t="s">
+        <v>182</v>
+      </c>
+      <c r="E30">
+        <v>25</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" t="s">
+        <v>93</v>
+      </c>
+      <c r="E31">
+        <v>20</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32">
+        <v>2</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D32" t="s">
+        <v>93</v>
+      </c>
+      <c r="E32">
+        <v>80</v>
+      </c>
+      <c r="F32">
+        <v>2</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>170</v>
+      </c>
+      <c r="B33">
+        <v>3</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33">
+        <v>90</v>
+      </c>
+      <c r="F33">
+        <v>2</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="D34" t="s">
+        <v>93</v>
+      </c>
+      <c r="E34">
+        <v>45</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>170</v>
+      </c>
+      <c r="B35">
+        <v>5</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D35" t="s">
+        <v>93</v>
+      </c>
+      <c r="E35">
+        <v>45</v>
+      </c>
+      <c r="F35">
+        <v>2</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B36">
+        <v>6</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D36" t="s">
+        <v>182</v>
+      </c>
+      <c r="E36">
+        <v>45</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>170</v>
+      </c>
+      <c r="B37">
+        <v>7</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D37" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37">
+        <v>60</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>170</v>
+      </c>
+      <c r="B38">
+        <v>8</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38">
+        <v>60</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>170</v>
+      </c>
+      <c r="B39">
+        <v>9</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39">
+        <v>80</v>
+      </c>
+      <c r="F39">
+        <v>3</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>170</v>
+      </c>
+      <c r="B40">
+        <v>10</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D40" t="s">
+        <v>93</v>
+      </c>
+      <c r="E40">
+        <v>80</v>
+      </c>
+      <c r="F40">
+        <v>3</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>170</v>
+      </c>
+      <c r="B41">
+        <v>11</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41">
+        <v>40</v>
+      </c>
+      <c r="F41">
+        <v>3</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>170</v>
+      </c>
+      <c r="B42">
+        <v>12</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D42" t="s">
+        <v>182</v>
+      </c>
+      <c r="E42">
+        <v>30</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43">
+        <v>13</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D43" t="s">
+        <v>93</v>
+      </c>
+      <c r="E43">
+        <v>45</v>
+      </c>
+      <c r="F43">
+        <v>2</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Jg6/Jg7 Zeitraum 2: Termine (Inputs/Coachings) eingetragen
18 Termine fuer Jg6, 22 fuer Jg7 aus den Kalendertabellen der PDFs,
21.09.-30.10.2026. Der "Paedagogische Tag" am 26.10. ist fuer beide
Jahrgaenge als normaler Termin (art: sonstiges) eingetragen, nicht als
Ferientag - Leo (24.09.2026): an dem Tag ist Heimarbeit angesagt, kein
Unterrichtsausfall, der Tag zaehlt weiter als Schultag.

Zwei kleine Abweichungen von der Vorlage, wo ein Feld nicht in eine
einzelne Zahl passte:
- Jg6, 06.10.: "Station 5,7" -> ein Termin mit beiden Nummern im Text,
  das Feld "station" nimmt nur eine Zahl.
- Jg6, 30.10.: "Station 13/14" -> genauso.

Im Browser gegengeprueft (Jg6 Woche 28.09.-02.10., Jg7 01.10. mit
Input+Coaching am selben Tag, "Paedagogischer Tag" zaehlt als
Schultag). Komplette Testsuite gruen.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg6.xlsx
+++ b/content/jahrgaenge/Jg6.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="328">
   <si>
     <t>Hinweise zu Jg6.xlsx</t>
   </si>
@@ -914,6 +914,96 @@
   </si>
   <si>
     <t>A2, A3, A4, Atlas, Wandkarte</t>
+  </si>
+  <si>
+    <t>2026-09-23</t>
+  </si>
+  <si>
+    <t>coaching</t>
+  </si>
+  <si>
+    <t>ADM</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
+  </si>
+  <si>
+    <t>HCO</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>Klimadiagramme auswerten</t>
+  </si>
+  <si>
+    <t>2026-09-29</t>
+  </si>
+  <si>
+    <t>DUB</t>
+  </si>
+  <si>
+    <t>Wiederholung Satzglieder erkennen</t>
+  </si>
+  <si>
+    <t>EPP</t>
+  </si>
+  <si>
+    <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>writing workshop</t>
+  </si>
+  <si>
+    <t>2026-10-05</t>
+  </si>
+  <si>
+    <t>2026-10-06</t>
+  </si>
+  <si>
+    <t>HS-NS erkennen, Satzbilder (Station 5 und 7)</t>
+  </si>
+  <si>
+    <t>2026-10-07</t>
+  </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
+    <t>Klimadiagramme zeichnen</t>
+  </si>
+  <si>
+    <t>2026-10-09</t>
+  </si>
+  <si>
+    <t>sonstiges</t>
+  </si>
+  <si>
+    <t>Pädagogischer Tag – Heimarbeit</t>
+  </si>
+  <si>
+    <t>2026-10-27</t>
+  </si>
+  <si>
+    <t>wörtliche Rede</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
+  </si>
+  <si>
+    <t>Topografie – wie arbeite ich mit Wandkarten</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>GEN – how to… (Station 13 und 14)</t>
   </si>
 </sst>
 </file>
@@ -5504,7 +5594,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" style="5" customWidth="1"/>
@@ -5546,6 +5636,582 @@
       </c>
       <c r="J1" s="3" t="s">
         <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="B2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="B3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>302</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="B4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D4" t="s">
+        <v>300</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="H4">
+        <v>9</v>
+      </c>
+      <c r="I4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" t="s">
+        <v>306</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B6" t="s">
+        <v>299</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>308</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="B7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>300</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" t="s">
+        <v>308</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
+      <c r="I8" t="s">
+        <v>8</v>
+      </c>
+      <c r="J8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>299</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>302</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" t="s">
+        <v>8</v>
+      </c>
+      <c r="I9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B10" t="s">
+        <v>299</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>300</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" t="s">
+        <v>8</v>
+      </c>
+      <c r="I10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="B11" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>306</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="H11" t="s">
+        <v>8</v>
+      </c>
+      <c r="I11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="B12" t="s">
+        <v>299</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>308</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" t="s">
+        <v>8</v>
+      </c>
+      <c r="I12" t="s">
+        <v>8</v>
+      </c>
+      <c r="J12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="B13" t="s">
+        <v>138</v>
+      </c>
+      <c r="C13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13" t="s">
+        <v>300</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="H13">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="B14" t="s">
+        <v>299</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>302</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" t="s">
+        <v>8</v>
+      </c>
+      <c r="I14" t="s">
+        <v>8</v>
+      </c>
+      <c r="J14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>319</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="H15" t="s">
+        <v>8</v>
+      </c>
+      <c r="I15" t="s">
+        <v>8</v>
+      </c>
+      <c r="J15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="B16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>306</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="H16">
+        <v>9</v>
+      </c>
+      <c r="I16" t="s">
+        <v>8</v>
+      </c>
+      <c r="J16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="B17" t="s">
+        <v>299</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>308</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" t="s">
+        <v>8</v>
+      </c>
+      <c r="I17" t="s">
+        <v>8</v>
+      </c>
+      <c r="J17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B18" t="s">
+        <v>138</v>
+      </c>
+      <c r="C18" t="s">
+        <v>171</v>
+      </c>
+      <c r="D18" t="s">
+        <v>300</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="H18" t="s">
+        <v>8</v>
+      </c>
+      <c r="I18" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B19" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" t="s">
+        <v>169</v>
+      </c>
+      <c r="D19" t="s">
+        <v>308</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="H19" t="s">
+        <v>8</v>
+      </c>
+      <c r="I19" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weihnachtsmarkt (18.12.) auch fuer Jg6/Jg7 eingetragen
Beim Gegenchecken aufgefallen: Jg5 hat fuer diese Woche schon eine
Sonderwoche ("Pufferwoche + SOUL Basics + Weihnachtsmarkt"), daher
dort keine separate Zeile noetig. Jg6 und Jg7 haben in der Woche aber
regulaeren Unterricht, dort fehlte der Weihnachtsmarkt komplett.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg6.xlsx
+++ b/content/jahrgaenge/Jg6.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2117" uniqueCount="475">
   <si>
     <t>Hinweise zu Jg6.xlsx</t>
   </si>
@@ -1172,6 +1172,12 @@
   </si>
   <si>
     <t>Viewing and listening skills</t>
+  </si>
+  <si>
+    <t>2026-12-18</t>
+  </si>
+  <si>
+    <t>Weihnachtsmarkt</t>
   </si>
   <si>
     <t>2027-01-04</t>
@@ -6029,7 +6035,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J122"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" style="5" customWidth="1"/>
@@ -8286,13 +8292,13 @@
         <v>384</v>
       </c>
       <c r="B71" t="s">
-        <v>138</v>
+        <v>342</v>
       </c>
       <c r="C71" t="s">
-        <v>171</v>
+        <v>8</v>
       </c>
       <c r="D71" t="s">
-        <v>300</v>
+        <v>8</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
@@ -8321,10 +8327,10 @@
         <v>138</v>
       </c>
       <c r="C72" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D72" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
@@ -8333,7 +8339,7 @@
         <v>8</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="H72" t="s">
         <v>8</v>
@@ -8347,16 +8353,16 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B73" t="s">
         <v>138</v>
       </c>
       <c r="C73" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D73" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E73" t="s">
         <v>8</v>
@@ -8365,10 +8371,10 @@
         <v>8</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="H73">
-        <v>9</v>
+        <v>369</v>
+      </c>
+      <c r="H73" t="s">
+        <v>8</v>
       </c>
       <c r="I73" t="s">
         <v>8</v>
@@ -8385,22 +8391,22 @@
         <v>138</v>
       </c>
       <c r="C74" t="s">
-        <v>44</v>
+        <v>169</v>
       </c>
       <c r="D74" t="s">
+        <v>304</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>8</v>
+      </c>
+      <c r="G74" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="E74" t="s">
-        <v>8</v>
-      </c>
-      <c r="F74" t="s">
-        <v>8</v>
-      </c>
-      <c r="G74" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="H74" t="s">
-        <v>8</v>
+      <c r="H74">
+        <v>9</v>
       </c>
       <c r="I74" t="s">
         <v>8</v>
@@ -8411,16 +8417,16 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B75" t="s">
         <v>138</v>
       </c>
       <c r="C75" t="s">
-        <v>166</v>
+        <v>44</v>
       </c>
       <c r="D75" t="s">
-        <v>302</v>
+        <v>392</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
@@ -8431,8 +8437,8 @@
       <c r="G75" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="H75">
-        <v>3</v>
+      <c r="H75" t="s">
+        <v>8</v>
       </c>
       <c r="I75" t="s">
         <v>8</v>
@@ -8449,22 +8455,22 @@
         <v>138</v>
       </c>
       <c r="C76" t="s">
-        <v>44</v>
+        <v>166</v>
       </c>
       <c r="D76" t="s">
+        <v>302</v>
+      </c>
+      <c r="E76" t="s">
+        <v>8</v>
+      </c>
+      <c r="F76" t="s">
+        <v>8</v>
+      </c>
+      <c r="G76" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="E76" t="s">
-        <v>8</v>
-      </c>
-      <c r="F76" t="s">
-        <v>8</v>
-      </c>
-      <c r="G76" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="H76" t="s">
-        <v>8</v>
+      <c r="H76">
+        <v>3</v>
       </c>
       <c r="I76" t="s">
         <v>8</v>
@@ -8475,16 +8481,16 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B77" t="s">
         <v>138</v>
       </c>
       <c r="C77" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="D77" t="s">
-        <v>358</v>
+        <v>397</v>
       </c>
       <c r="E77" t="s">
         <v>8</v>
@@ -8495,8 +8501,8 @@
       <c r="G77" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="H77">
-        <v>5</v>
+      <c r="H77" t="s">
+        <v>8</v>
       </c>
       <c r="I77" t="s">
         <v>8</v>
@@ -8513,10 +8519,10 @@
         <v>138</v>
       </c>
       <c r="C78" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="D78" t="s">
-        <v>390</v>
+        <v>358</v>
       </c>
       <c r="E78" t="s">
         <v>8</v>
@@ -8527,8 +8533,8 @@
       <c r="G78" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="H78" t="s">
-        <v>8</v>
+      <c r="H78">
+        <v>5</v>
       </c>
       <c r="I78" t="s">
         <v>8</v>
@@ -8545,10 +8551,10 @@
         <v>138</v>
       </c>
       <c r="C79" t="s">
-        <v>166</v>
+        <v>44</v>
       </c>
       <c r="D79" t="s">
-        <v>302</v>
+        <v>392</v>
       </c>
       <c r="E79" t="s">
         <v>8</v>
@@ -8559,8 +8565,8 @@
       <c r="G79" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="H79">
-        <v>5</v>
+      <c r="H79" t="s">
+        <v>8</v>
       </c>
       <c r="I79" t="s">
         <v>8</v>
@@ -8577,10 +8583,10 @@
         <v>138</v>
       </c>
       <c r="C80" t="s">
-        <v>44</v>
+        <v>166</v>
       </c>
       <c r="D80" t="s">
-        <v>395</v>
+        <v>302</v>
       </c>
       <c r="E80" t="s">
         <v>8</v>
@@ -8589,10 +8595,10 @@
         <v>8</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="H80" t="s">
-        <v>8</v>
+        <v>404</v>
+      </c>
+      <c r="H80">
+        <v>5</v>
       </c>
       <c r="I80" t="s">
         <v>8</v>
@@ -8603,16 +8609,16 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B81" t="s">
         <v>138</v>
       </c>
       <c r="C81" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="D81" t="s">
-        <v>358</v>
+        <v>397</v>
       </c>
       <c r="E81" t="s">
         <v>8</v>
@@ -8623,8 +8629,8 @@
       <c r="G81" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="H81">
-        <v>5</v>
+      <c r="H81" t="s">
+        <v>8</v>
       </c>
       <c r="I81" t="s">
         <v>8</v>
@@ -8635,16 +8641,16 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B82" t="s">
-        <v>342</v>
+        <v>138</v>
       </c>
       <c r="C82" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="D82" t="s">
-        <v>8</v>
+        <v>358</v>
       </c>
       <c r="E82" t="s">
         <v>8</v>
@@ -8653,10 +8659,10 @@
         <v>8</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="H82" t="s">
-        <v>8</v>
+        <v>400</v>
+      </c>
+      <c r="H82">
+        <v>5</v>
       </c>
       <c r="I82" t="s">
         <v>8</v>
@@ -8667,16 +8673,16 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B83" t="s">
-        <v>138</v>
+        <v>342</v>
       </c>
       <c r="C83" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="D83" t="s">
-        <v>390</v>
+        <v>8</v>
       </c>
       <c r="E83" t="s">
         <v>8</v>
@@ -8685,10 +8691,10 @@
         <v>8</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="H83">
-        <v>18</v>
+        <v>343</v>
+      </c>
+      <c r="H83" t="s">
+        <v>8</v>
       </c>
       <c r="I83" t="s">
         <v>8</v>
@@ -8705,10 +8711,10 @@
         <v>138</v>
       </c>
       <c r="C84" t="s">
-        <v>166</v>
+        <v>44</v>
       </c>
       <c r="D84" t="s">
-        <v>302</v>
+        <v>392</v>
       </c>
       <c r="E84" t="s">
         <v>8</v>
@@ -8720,7 +8726,7 @@
         <v>409</v>
       </c>
       <c r="H84">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="I84" t="s">
         <v>8</v>
@@ -8737,10 +8743,10 @@
         <v>138</v>
       </c>
       <c r="C85" t="s">
-        <v>44</v>
+        <v>166</v>
       </c>
       <c r="D85" t="s">
-        <v>395</v>
+        <v>302</v>
       </c>
       <c r="E85" t="s">
         <v>8</v>
@@ -8749,9 +8755,9 @@
         <v>8</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="H85" t="s">
+        <v>411</v>
+      </c>
+      <c r="H85">
         <v>8</v>
       </c>
       <c r="I85" t="s">
@@ -8763,16 +8769,16 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B86" t="s">
         <v>138</v>
       </c>
       <c r="C86" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="D86" t="s">
-        <v>358</v>
+        <v>397</v>
       </c>
       <c r="E86" t="s">
         <v>8</v>
@@ -8783,8 +8789,8 @@
       <c r="G86" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="H86">
-        <v>5</v>
+      <c r="H86" t="s">
+        <v>8</v>
       </c>
       <c r="I86" t="s">
         <v>8</v>
@@ -8795,16 +8801,16 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B87" t="s">
         <v>138</v>
       </c>
       <c r="C87" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="D87" t="s">
-        <v>300</v>
+        <v>358</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
@@ -8813,10 +8819,10 @@
         <v>8</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>413</v>
+        <v>400</v>
       </c>
       <c r="H87">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I87" t="s">
         <v>8</v>
@@ -8833,10 +8839,10 @@
         <v>138</v>
       </c>
       <c r="C88" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D88" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="E88" t="s">
         <v>8</v>
@@ -8865,10 +8871,10 @@
         <v>138</v>
       </c>
       <c r="C89" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="D89" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E89" t="s">
         <v>8</v>
@@ -8880,7 +8886,7 @@
         <v>417</v>
       </c>
       <c r="H89">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I89" t="s">
         <v>8</v>
@@ -8897,10 +8903,10 @@
         <v>138</v>
       </c>
       <c r="C90" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="D90" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="E90" t="s">
         <v>8</v>
@@ -8911,8 +8917,8 @@
       <c r="G90" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="H90" t="s">
-        <v>8</v>
+      <c r="H90">
+        <v>6</v>
       </c>
       <c r="I90" t="s">
         <v>8</v>
@@ -8929,10 +8935,10 @@
         <v>138</v>
       </c>
       <c r="C91" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D91" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="E91" t="s">
         <v>8</v>
@@ -8943,8 +8949,8 @@
       <c r="G91" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="H91">
-        <v>5</v>
+      <c r="H91" t="s">
+        <v>8</v>
       </c>
       <c r="I91" t="s">
         <v>8</v>
@@ -8961,10 +8967,10 @@
         <v>138</v>
       </c>
       <c r="C92" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="D92" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E92" t="s">
         <v>8</v>
@@ -8975,8 +8981,8 @@
       <c r="G92" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="H92" t="s">
-        <v>8</v>
+      <c r="H92">
+        <v>5</v>
       </c>
       <c r="I92" t="s">
         <v>8</v>
@@ -8993,10 +8999,10 @@
         <v>138</v>
       </c>
       <c r="C93" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="D93" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="E93" t="s">
         <v>8</v>
@@ -9007,8 +9013,8 @@
       <c r="G93" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="H93">
-        <v>4</v>
+      <c r="H93" t="s">
+        <v>8</v>
       </c>
       <c r="I93" t="s">
         <v>8</v>
@@ -9025,10 +9031,10 @@
         <v>138</v>
       </c>
       <c r="C94" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D94" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="E94" t="s">
         <v>8</v>
@@ -9037,10 +9043,10 @@
         <v>8</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="H94">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I94" t="s">
         <v>8</v>
@@ -9051,16 +9057,16 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B95" t="s">
         <v>138</v>
       </c>
       <c r="C95" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="D95" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E95" t="s">
         <v>8</v>
@@ -9071,8 +9077,8 @@
       <c r="G95" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="H95" t="s">
-        <v>8</v>
+      <c r="H95">
+        <v>5</v>
       </c>
       <c r="I95" t="s">
         <v>8</v>
@@ -9083,16 +9089,16 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B96" t="s">
         <v>138</v>
       </c>
       <c r="C96" t="s">
-        <v>166</v>
+        <v>72</v>
       </c>
       <c r="D96" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E96" t="s">
         <v>8</v>
@@ -9101,10 +9107,10 @@
         <v>8</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="H96">
-        <v>6</v>
+        <v>425</v>
+      </c>
+      <c r="H96" t="s">
+        <v>8</v>
       </c>
       <c r="I96" t="s">
         <v>8</v>
@@ -9118,13 +9124,13 @@
         <v>430</v>
       </c>
       <c r="B97" t="s">
-        <v>342</v>
+        <v>138</v>
       </c>
       <c r="C97" t="s">
-        <v>8</v>
+        <v>166</v>
       </c>
       <c r="D97" t="s">
-        <v>8</v>
+        <v>302</v>
       </c>
       <c r="E97" t="s">
         <v>8</v>
@@ -9133,10 +9139,10 @@
         <v>8</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="H97" t="s">
-        <v>8</v>
+        <v>431</v>
+      </c>
+      <c r="H97">
+        <v>6</v>
       </c>
       <c r="I97" t="s">
         <v>8</v>
@@ -9147,16 +9153,16 @@
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B98" t="s">
-        <v>138</v>
+        <v>342</v>
       </c>
       <c r="C98" t="s">
-        <v>169</v>
+        <v>8</v>
       </c>
       <c r="D98" t="s">
-        <v>304</v>
+        <v>8</v>
       </c>
       <c r="E98" t="s">
         <v>8</v>
@@ -9165,10 +9171,10 @@
         <v>8</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="H98">
-        <v>1</v>
+        <v>343</v>
+      </c>
+      <c r="H98" t="s">
+        <v>8</v>
       </c>
       <c r="I98" t="s">
         <v>8</v>
@@ -9185,10 +9191,10 @@
         <v>138</v>
       </c>
       <c r="C99" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="D99" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E99" t="s">
         <v>8</v>
@@ -9199,8 +9205,8 @@
       <c r="G99" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="H99" t="s">
-        <v>8</v>
+      <c r="H99">
+        <v>1</v>
       </c>
       <c r="I99" t="s">
         <v>8</v>
@@ -9217,10 +9223,10 @@
         <v>138</v>
       </c>
       <c r="C100" t="s">
-        <v>166</v>
+        <v>72</v>
       </c>
       <c r="D100" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E100" t="s">
         <v>8</v>
@@ -9231,7 +9237,7 @@
       <c r="G100" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="H100">
+      <c r="H100" t="s">
         <v>8</v>
       </c>
       <c r="I100" t="s">
@@ -9249,10 +9255,10 @@
         <v>138</v>
       </c>
       <c r="C101" t="s">
-        <v>72</v>
+        <v>166</v>
       </c>
       <c r="D101" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="E101" t="s">
         <v>8</v>
@@ -9281,10 +9287,10 @@
         <v>138</v>
       </c>
       <c r="C102" t="s">
-        <v>169</v>
+        <v>72</v>
       </c>
       <c r="D102" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E102" t="s">
         <v>8</v>
@@ -9296,7 +9302,7 @@
         <v>440</v>
       </c>
       <c r="H102">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I102" t="s">
         <v>8</v>
@@ -9310,13 +9316,13 @@
         <v>441</v>
       </c>
       <c r="B103" t="s">
-        <v>342</v>
+        <v>138</v>
       </c>
       <c r="C103" t="s">
-        <v>8</v>
+        <v>169</v>
       </c>
       <c r="D103" t="s">
-        <v>8</v>
+        <v>304</v>
       </c>
       <c r="E103" t="s">
         <v>8</v>
@@ -9327,8 +9333,8 @@
       <c r="G103" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="H103" t="s">
-        <v>8</v>
+      <c r="H103">
+        <v>5</v>
       </c>
       <c r="I103" t="s">
         <v>8</v>
@@ -9342,13 +9348,13 @@
         <v>443</v>
       </c>
       <c r="B104" t="s">
-        <v>138</v>
+        <v>342</v>
       </c>
       <c r="C104" t="s">
-        <v>166</v>
+        <v>8</v>
       </c>
       <c r="D104" t="s">
-        <v>302</v>
+        <v>8</v>
       </c>
       <c r="E104" t="s">
         <v>8</v>
@@ -9359,8 +9365,8 @@
       <c r="G104" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="H104">
-        <v>11</v>
+      <c r="H104" t="s">
+        <v>8</v>
       </c>
       <c r="I104" t="s">
         <v>8</v>
@@ -9377,10 +9383,10 @@
         <v>138</v>
       </c>
       <c r="C105" t="s">
-        <v>72</v>
+        <v>166</v>
       </c>
       <c r="D105" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="E105" t="s">
         <v>8</v>
@@ -9392,7 +9398,7 @@
         <v>446</v>
       </c>
       <c r="H105">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I105" t="s">
         <v>8</v>
@@ -9409,10 +9415,10 @@
         <v>138</v>
       </c>
       <c r="C106" t="s">
-        <v>169</v>
+        <v>72</v>
       </c>
       <c r="D106" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E106" t="s">
         <v>8</v>
@@ -9424,7 +9430,7 @@
         <v>448</v>
       </c>
       <c r="H106">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I106" t="s">
         <v>8</v>
@@ -9453,10 +9459,10 @@
         <v>8</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>432</v>
+        <v>450</v>
       </c>
       <c r="H107">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I107" t="s">
         <v>8</v>
@@ -9467,16 +9473,16 @@
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B108" t="s">
         <v>138</v>
       </c>
       <c r="C108" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D108" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="E108" t="s">
         <v>8</v>
@@ -9485,10 +9491,10 @@
         <v>8</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="H108" t="s">
-        <v>8</v>
+        <v>434</v>
+      </c>
+      <c r="H108">
+        <v>1</v>
       </c>
       <c r="I108" t="s">
         <v>8</v>
@@ -9505,22 +9511,22 @@
         <v>138</v>
       </c>
       <c r="C109" t="s">
-        <v>44</v>
+        <v>171</v>
       </c>
       <c r="D109" t="s">
+        <v>300</v>
+      </c>
+      <c r="E109" t="s">
+        <v>8</v>
+      </c>
+      <c r="F109" t="s">
+        <v>8</v>
+      </c>
+      <c r="G109" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="E109" t="s">
-        <v>8</v>
-      </c>
-      <c r="F109" t="s">
-        <v>8</v>
-      </c>
-      <c r="G109" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="H109">
-        <v>7</v>
+      <c r="H109" t="s">
+        <v>8</v>
       </c>
       <c r="I109" t="s">
         <v>8</v>
@@ -9531,7 +9537,7 @@
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B110" t="s">
         <v>138</v>
@@ -9540,7 +9546,7 @@
         <v>44</v>
       </c>
       <c r="D110" t="s">
-        <v>395</v>
+        <v>455</v>
       </c>
       <c r="E110" t="s">
         <v>8</v>
@@ -9552,7 +9558,7 @@
         <v>456</v>
       </c>
       <c r="H110">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I110" t="s">
         <v>8</v>
@@ -9569,10 +9575,10 @@
         <v>138</v>
       </c>
       <c r="C111" t="s">
-        <v>171</v>
+        <v>44</v>
       </c>
       <c r="D111" t="s">
-        <v>300</v>
+        <v>397</v>
       </c>
       <c r="E111" t="s">
         <v>8</v>
@@ -9583,7 +9589,7 @@
       <c r="G111" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="H111" t="s">
+      <c r="H111">
         <v>8</v>
       </c>
       <c r="I111" t="s">
@@ -9601,10 +9607,10 @@
         <v>138</v>
       </c>
       <c r="C112" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D112" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="E112" t="s">
         <v>8</v>
@@ -9613,10 +9619,10 @@
         <v>8</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="H112">
-        <v>5</v>
+        <v>460</v>
+      </c>
+      <c r="H112" t="s">
+        <v>8</v>
       </c>
       <c r="I112" t="s">
         <v>8</v>
@@ -9627,16 +9633,16 @@
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B113" t="s">
         <v>138</v>
       </c>
       <c r="C113" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D113" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="E113" t="s">
         <v>8</v>
@@ -9645,10 +9651,10 @@
         <v>8</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="H113" t="s">
-        <v>8</v>
+        <v>442</v>
+      </c>
+      <c r="H113">
+        <v>5</v>
       </c>
       <c r="I113" t="s">
         <v>8</v>
@@ -9659,16 +9665,16 @@
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B114" t="s">
         <v>138</v>
       </c>
       <c r="C114" t="s">
-        <v>44</v>
+        <v>171</v>
       </c>
       <c r="D114" t="s">
-        <v>453</v>
+        <v>300</v>
       </c>
       <c r="E114" t="s">
         <v>8</v>
@@ -9677,7 +9683,7 @@
         <v>8</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="H114" t="s">
         <v>8</v>
@@ -9697,10 +9703,10 @@
         <v>138</v>
       </c>
       <c r="C115" t="s">
-        <v>169</v>
+        <v>44</v>
       </c>
       <c r="D115" t="s">
-        <v>304</v>
+        <v>455</v>
       </c>
       <c r="E115" t="s">
         <v>8</v>
@@ -9709,10 +9715,10 @@
         <v>8</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="H115">
-        <v>6</v>
+        <v>464</v>
+      </c>
+      <c r="H115" t="s">
+        <v>8</v>
       </c>
       <c r="I115" t="s">
         <v>8</v>
@@ -9723,16 +9729,16 @@
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B116" t="s">
         <v>138</v>
       </c>
       <c r="C116" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D116" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E116" t="s">
         <v>8</v>
@@ -9741,10 +9747,10 @@
         <v>8</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H116" t="s">
-        <v>8</v>
+        <v>450</v>
+      </c>
+      <c r="H116">
+        <v>6</v>
       </c>
       <c r="I116" t="s">
         <v>8</v>
@@ -9755,16 +9761,16 @@
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B117" t="s">
         <v>138</v>
       </c>
       <c r="C117" t="s">
-        <v>72</v>
+        <v>166</v>
       </c>
       <c r="D117" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="E117" t="s">
         <v>8</v>
@@ -9787,16 +9793,16 @@
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B118" t="s">
         <v>138</v>
       </c>
       <c r="C118" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="D118" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E118" t="s">
         <v>8</v>
@@ -9805,7 +9811,7 @@
         <v>8</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>467</v>
+        <v>8</v>
       </c>
       <c r="H118" t="s">
         <v>8</v>
@@ -9857,10 +9863,10 @@
         <v>138</v>
       </c>
       <c r="C120" t="s">
-        <v>171</v>
+        <v>44</v>
       </c>
       <c r="D120" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="E120" t="s">
         <v>8</v>
@@ -9889,27 +9895,59 @@
         <v>138</v>
       </c>
       <c r="C121" t="s">
+        <v>171</v>
+      </c>
+      <c r="D121" t="s">
+        <v>300</v>
+      </c>
+      <c r="E121" t="s">
+        <v>8</v>
+      </c>
+      <c r="F121" t="s">
+        <v>8</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="H121" t="s">
+        <v>8</v>
+      </c>
+      <c r="I121" t="s">
+        <v>8</v>
+      </c>
+      <c r="J121" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B122" t="s">
+        <v>138</v>
+      </c>
+      <c r="C122" t="s">
         <v>169</v>
       </c>
-      <c r="D121" t="s">
+      <c r="D122" t="s">
         <v>304</v>
       </c>
-      <c r="E121" t="s">
-        <v>8</v>
-      </c>
-      <c r="F121" t="s">
-        <v>8</v>
-      </c>
-      <c r="G121" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H121" t="s">
-        <v>8</v>
-      </c>
-      <c r="I121" t="s">
-        <v>8</v>
-      </c>
-      <c r="J121" t="s">
+      <c r="E122" t="s">
+        <v>8</v>
+      </c>
+      <c r="F122" t="s">
+        <v>8</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H122" t="s">
+        <v>8</v>
+      </c>
+      <c r="I122" t="s">
+        <v>8</v>
+      </c>
+      <c r="J122" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Jg6 "Unter der Lupe": echte Mikroskopier-Themen statt Platzhalter
Leo (29.09.2026) bestaetigt: pro Klasse (6A/6B/6C) zwei Pflichtinputs,
zuerst "Mikroskopieren: Einführung" (HAM), dann "Mikroskopieren:
Zwiebelhäutchen" (BRU) - ersetzt die sechs "6X: xxx"-Platzhalter aus
dem Quelldokument.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg6.xlsx
+++ b/content/jahrgaenge/Jg6.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2117" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2117" uniqueCount="477">
   <si>
     <t>Hinweise zu Jg6.xlsx</t>
   </si>
@@ -1078,6 +1078,9 @@
     <t>2026-11-09</t>
   </si>
   <si>
+    <t>Mikroskopieren: Einführung</t>
+  </si>
+  <si>
     <t>2026-11-10</t>
   </si>
   <si>
@@ -1100,6 +1103,9 @@
   </si>
   <si>
     <t>2026-11-13</t>
+  </si>
+  <si>
+    <t>Mikroskopieren: Zwiebelhäutchen</t>
   </si>
   <si>
     <t>2026-11-16</t>
@@ -7443,7 +7449,7 @@
         <v>8</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>8</v>
+        <v>352</v>
       </c>
       <c r="H44" t="s">
         <v>8</v>
@@ -7457,7 +7463,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B45" t="s">
         <v>138</v>
@@ -7466,7 +7472,7 @@
         <v>44</v>
       </c>
       <c r="D45" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E45" t="s">
         <v>8</v>
@@ -7475,7 +7481,7 @@
         <v>8</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="H45" t="s">
         <v>8</v>
@@ -7489,7 +7495,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B46" t="s">
         <v>299</v>
@@ -7521,7 +7527,7 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B47" t="s">
         <v>138</v>
@@ -7539,7 +7545,7 @@
         <v>8</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H47">
         <v>11</v>
@@ -7553,7 +7559,7 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B48" t="s">
         <v>299</v>
@@ -7585,7 +7591,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B49" t="s">
         <v>299</v>
@@ -7594,7 +7600,7 @@
         <v>8</v>
       </c>
       <c r="D49" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
@@ -7617,7 +7623,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B50" t="s">
         <v>138</v>
@@ -7635,7 +7641,7 @@
         <v>8</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>8</v>
+        <v>361</v>
       </c>
       <c r="H50" t="s">
         <v>8</v>
@@ -7649,7 +7655,7 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B51" t="s">
         <v>138</v>
@@ -7667,7 +7673,7 @@
         <v>8</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>8</v>
+        <v>352</v>
       </c>
       <c r="H51" t="s">
         <v>8</v>
@@ -7681,7 +7687,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B52" t="s">
         <v>138</v>
@@ -7690,7 +7696,7 @@
         <v>44</v>
       </c>
       <c r="D52" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E52" t="s">
         <v>8</v>
@@ -7699,7 +7705,7 @@
         <v>8</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="H52">
         <v>5</v>
@@ -7713,7 +7719,7 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B53" t="s">
         <v>299</v>
@@ -7745,7 +7751,7 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B54" t="s">
         <v>299</v>
@@ -7754,7 +7760,7 @@
         <v>8</v>
       </c>
       <c r="D54" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E54" t="s">
         <v>8</v>
@@ -7777,7 +7783,7 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B55" t="s">
         <v>138</v>
@@ -7795,7 +7801,7 @@
         <v>8</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>8</v>
+        <v>361</v>
       </c>
       <c r="H55" t="s">
         <v>8</v>
@@ -7809,7 +7815,7 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B56" t="s">
         <v>138</v>
@@ -7827,7 +7833,7 @@
         <v>8</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>8</v>
+        <v>352</v>
       </c>
       <c r="H56" t="s">
         <v>8</v>
@@ -7841,7 +7847,7 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B57" t="s">
         <v>138</v>
@@ -7850,7 +7856,7 @@
         <v>44</v>
       </c>
       <c r="D57" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E57" t="s">
         <v>8</v>
@@ -7859,7 +7865,7 @@
         <v>8</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="H57" t="s">
         <v>8</v>
@@ -7873,7 +7879,7 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B58" t="s">
         <v>138</v>
@@ -7891,7 +7897,7 @@
         <v>8</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="H58" t="s">
         <v>8</v>
@@ -7905,7 +7911,7 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B59" t="s">
         <v>299</v>
@@ -7937,7 +7943,7 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B60" t="s">
         <v>299</v>
@@ -7946,7 +7952,7 @@
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E60" t="s">
         <v>8</v>
@@ -7969,7 +7975,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B61" t="s">
         <v>138</v>
@@ -7987,7 +7993,7 @@
         <v>8</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>8</v>
+        <v>361</v>
       </c>
       <c r="H61" t="s">
         <v>8</v>
@@ -8001,7 +8007,7 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B62" t="s">
         <v>299</v>
@@ -8033,7 +8039,7 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B63" t="s">
         <v>299</v>
@@ -8065,7 +8071,7 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B64" t="s">
         <v>138</v>
@@ -8083,7 +8089,7 @@
         <v>8</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="H64">
         <v>5</v>
@@ -8097,7 +8103,7 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B65" t="s">
         <v>138</v>
@@ -8129,7 +8135,7 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B66" t="s">
         <v>138</v>
@@ -8147,7 +8153,7 @@
         <v>8</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="H66">
         <v>2</v>
@@ -8161,7 +8167,7 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B67" t="s">
         <v>138</v>
@@ -8179,7 +8185,7 @@
         <v>8</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="H67">
         <v>7</v>
@@ -8193,7 +8199,7 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B68" t="s">
         <v>299</v>
@@ -8225,7 +8231,7 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B69" t="s">
         <v>138</v>
@@ -8243,7 +8249,7 @@
         <v>8</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H69">
         <v>11</v>
@@ -8257,7 +8263,7 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B70" t="s">
         <v>138</v>
@@ -8275,7 +8281,7 @@
         <v>8</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="H70">
         <v>8</v>
@@ -8289,7 +8295,7 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B71" t="s">
         <v>342</v>
@@ -8307,7 +8313,7 @@
         <v>8</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="H71" t="s">
         <v>8</v>
@@ -8321,7 +8327,7 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B72" t="s">
         <v>138</v>
@@ -8339,7 +8345,7 @@
         <v>8</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H72" t="s">
         <v>8</v>
@@ -8353,7 +8359,7 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B73" t="s">
         <v>138</v>
@@ -8371,7 +8377,7 @@
         <v>8</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="H73" t="s">
         <v>8</v>
@@ -8385,7 +8391,7 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B74" t="s">
         <v>138</v>
@@ -8403,7 +8409,7 @@
         <v>8</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="H74">
         <v>9</v>
@@ -8417,7 +8423,7 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B75" t="s">
         <v>138</v>
@@ -8426,7 +8432,7 @@
         <v>44</v>
       </c>
       <c r="D75" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
@@ -8435,7 +8441,7 @@
         <v>8</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="H75" t="s">
         <v>8</v>
@@ -8449,7 +8455,7 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B76" t="s">
         <v>138</v>
@@ -8467,7 +8473,7 @@
         <v>8</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="H76">
         <v>3</v>
@@ -8481,7 +8487,7 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B77" t="s">
         <v>138</v>
@@ -8490,7 +8496,7 @@
         <v>44</v>
       </c>
       <c r="D77" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E77" t="s">
         <v>8</v>
@@ -8499,7 +8505,7 @@
         <v>8</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="H77" t="s">
         <v>8</v>
@@ -8513,7 +8519,7 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B78" t="s">
         <v>138</v>
@@ -8522,7 +8528,7 @@
         <v>72</v>
       </c>
       <c r="D78" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E78" t="s">
         <v>8</v>
@@ -8531,7 +8537,7 @@
         <v>8</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="H78">
         <v>5</v>
@@ -8545,7 +8551,7 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B79" t="s">
         <v>138</v>
@@ -8554,7 +8560,7 @@
         <v>44</v>
       </c>
       <c r="D79" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E79" t="s">
         <v>8</v>
@@ -8563,7 +8569,7 @@
         <v>8</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H79" t="s">
         <v>8</v>
@@ -8577,7 +8583,7 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B80" t="s">
         <v>138</v>
@@ -8595,7 +8601,7 @@
         <v>8</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="H80">
         <v>5</v>
@@ -8609,7 +8615,7 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B81" t="s">
         <v>138</v>
@@ -8618,7 +8624,7 @@
         <v>44</v>
       </c>
       <c r="D81" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E81" t="s">
         <v>8</v>
@@ -8627,7 +8633,7 @@
         <v>8</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="H81" t="s">
         <v>8</v>
@@ -8641,7 +8647,7 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B82" t="s">
         <v>138</v>
@@ -8650,7 +8656,7 @@
         <v>72</v>
       </c>
       <c r="D82" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E82" t="s">
         <v>8</v>
@@ -8659,7 +8665,7 @@
         <v>8</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="H82">
         <v>5</v>
@@ -8673,7 +8679,7 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B83" t="s">
         <v>342</v>
@@ -8705,7 +8711,7 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B84" t="s">
         <v>138</v>
@@ -8714,7 +8720,7 @@
         <v>44</v>
       </c>
       <c r="D84" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E84" t="s">
         <v>8</v>
@@ -8723,7 +8729,7 @@
         <v>8</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="H84">
         <v>18</v>
@@ -8737,7 +8743,7 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B85" t="s">
         <v>138</v>
@@ -8755,7 +8761,7 @@
         <v>8</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="H85">
         <v>8</v>
@@ -8769,7 +8775,7 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B86" t="s">
         <v>138</v>
@@ -8778,7 +8784,7 @@
         <v>44</v>
       </c>
       <c r="D86" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E86" t="s">
         <v>8</v>
@@ -8787,7 +8793,7 @@
         <v>8</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="H86" t="s">
         <v>8</v>
@@ -8801,7 +8807,7 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B87" t="s">
         <v>138</v>
@@ -8810,7 +8816,7 @@
         <v>72</v>
       </c>
       <c r="D87" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
@@ -8819,7 +8825,7 @@
         <v>8</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="H87">
         <v>5</v>
@@ -8833,7 +8839,7 @@
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B88" t="s">
         <v>138</v>
@@ -8851,7 +8857,7 @@
         <v>8</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="H88">
         <v>2</v>
@@ -8865,7 +8871,7 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B89" t="s">
         <v>138</v>
@@ -8883,7 +8889,7 @@
         <v>8</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="H89">
         <v>2</v>
@@ -8897,7 +8903,7 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B90" t="s">
         <v>138</v>
@@ -8915,7 +8921,7 @@
         <v>8</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="H90">
         <v>6</v>
@@ -8929,7 +8935,7 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B91" t="s">
         <v>138</v>
@@ -8947,7 +8953,7 @@
         <v>8</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="H91" t="s">
         <v>8</v>
@@ -8961,7 +8967,7 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B92" t="s">
         <v>138</v>
@@ -8979,7 +8985,7 @@
         <v>8</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="H92">
         <v>5</v>
@@ -8993,7 +8999,7 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B93" t="s">
         <v>138</v>
@@ -9011,7 +9017,7 @@
         <v>8</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="H93" t="s">
         <v>8</v>
@@ -9025,7 +9031,7 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B94" t="s">
         <v>138</v>
@@ -9043,7 +9049,7 @@
         <v>8</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="H94">
         <v>4</v>
@@ -9057,7 +9063,7 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B95" t="s">
         <v>138</v>
@@ -9075,7 +9081,7 @@
         <v>8</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="H95">
         <v>5</v>
@@ -9089,7 +9095,7 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B96" t="s">
         <v>138</v>
@@ -9107,7 +9113,7 @@
         <v>8</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="H96" t="s">
         <v>8</v>
@@ -9121,7 +9127,7 @@
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B97" t="s">
         <v>138</v>
@@ -9139,7 +9145,7 @@
         <v>8</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="H97">
         <v>6</v>
@@ -9153,7 +9159,7 @@
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B98" t="s">
         <v>342</v>
@@ -9185,7 +9191,7 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B99" t="s">
         <v>138</v>
@@ -9203,7 +9209,7 @@
         <v>8</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="H99">
         <v>1</v>
@@ -9217,7 +9223,7 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B100" t="s">
         <v>138</v>
@@ -9235,7 +9241,7 @@
         <v>8</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H100" t="s">
         <v>8</v>
@@ -9249,7 +9255,7 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B101" t="s">
         <v>138</v>
@@ -9267,7 +9273,7 @@
         <v>8</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="H101">
         <v>8</v>
@@ -9281,7 +9287,7 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B102" t="s">
         <v>138</v>
@@ -9299,7 +9305,7 @@
         <v>8</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H102">
         <v>8</v>
@@ -9313,7 +9319,7 @@
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B103" t="s">
         <v>138</v>
@@ -9331,7 +9337,7 @@
         <v>8</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="H103">
         <v>5</v>
@@ -9345,7 +9351,7 @@
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B104" t="s">
         <v>342</v>
@@ -9363,7 +9369,7 @@
         <v>8</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="H104" t="s">
         <v>8</v>
@@ -9377,7 +9383,7 @@
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B105" t="s">
         <v>138</v>
@@ -9395,7 +9401,7 @@
         <v>8</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H105">
         <v>11</v>
@@ -9409,7 +9415,7 @@
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B106" t="s">
         <v>138</v>
@@ -9427,7 +9433,7 @@
         <v>8</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="H106">
         <v>10</v>
@@ -9441,7 +9447,7 @@
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B107" t="s">
         <v>138</v>
@@ -9459,7 +9465,7 @@
         <v>8</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="H107">
         <v>6</v>
@@ -9473,7 +9479,7 @@
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B108" t="s">
         <v>138</v>
@@ -9491,7 +9497,7 @@
         <v>8</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="H108">
         <v>1</v>
@@ -9505,7 +9511,7 @@
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B109" t="s">
         <v>138</v>
@@ -9523,7 +9529,7 @@
         <v>8</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="H109" t="s">
         <v>8</v>
@@ -9537,7 +9543,7 @@
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B110" t="s">
         <v>138</v>
@@ -9546,7 +9552,7 @@
         <v>44</v>
       </c>
       <c r="D110" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E110" t="s">
         <v>8</v>
@@ -9555,7 +9561,7 @@
         <v>8</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="H110">
         <v>7</v>
@@ -9569,7 +9575,7 @@
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B111" t="s">
         <v>138</v>
@@ -9578,7 +9584,7 @@
         <v>44</v>
       </c>
       <c r="D111" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E111" t="s">
         <v>8</v>
@@ -9587,7 +9593,7 @@
         <v>8</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="H111">
         <v>8</v>
@@ -9601,7 +9607,7 @@
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B112" t="s">
         <v>138</v>
@@ -9619,7 +9625,7 @@
         <v>8</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="H112" t="s">
         <v>8</v>
@@ -9633,7 +9639,7 @@
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B113" t="s">
         <v>138</v>
@@ -9651,7 +9657,7 @@
         <v>8</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="H113">
         <v>5</v>
@@ -9665,7 +9671,7 @@
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B114" t="s">
         <v>138</v>
@@ -9683,7 +9689,7 @@
         <v>8</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="H114" t="s">
         <v>8</v>
@@ -9697,7 +9703,7 @@
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B115" t="s">
         <v>138</v>
@@ -9706,7 +9712,7 @@
         <v>44</v>
       </c>
       <c r="D115" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E115" t="s">
         <v>8</v>
@@ -9715,7 +9721,7 @@
         <v>8</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="H115" t="s">
         <v>8</v>
@@ -9729,7 +9735,7 @@
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B116" t="s">
         <v>138</v>
@@ -9747,7 +9753,7 @@
         <v>8</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="H116">
         <v>6</v>
@@ -9761,7 +9767,7 @@
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B117" t="s">
         <v>138</v>
@@ -9793,7 +9799,7 @@
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B118" t="s">
         <v>138</v>
@@ -9825,7 +9831,7 @@
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" s="5" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B119" t="s">
         <v>138</v>
@@ -9843,7 +9849,7 @@
         <v>8</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="H119" t="s">
         <v>8</v>
@@ -9857,7 +9863,7 @@
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B120" t="s">
         <v>138</v>
@@ -9875,7 +9881,7 @@
         <v>8</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="H120" t="s">
         <v>8</v>
@@ -9889,7 +9895,7 @@
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B121" t="s">
         <v>138</v>
@@ -9907,7 +9913,7 @@
         <v>8</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="H121" t="s">
         <v>8</v>
@@ -9921,7 +9927,7 @@
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B122" t="s">
         <v>138</v>

</xml_diff>